<commit_message>
#49 (Quantity Per Board) Column name Updated.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Control-Board/PCBWay_BOM-Control-Board.xlsx
+++ b/Deliverables/BOM/Control-Board/PCBWay_BOM-Control-Board.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ManarHarake-sEMGDevice\Deliverables\BOM\Control-Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{575E30EA-9A14-4D3C-A37C-BCE36693EABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C26CC9F6-51D2-407A-B8BE-31117E0FF244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="11790" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -680,9 +680,6 @@
     <t>C86816</t>
   </si>
   <si>
-    <t>Quantity (1 Board)</t>
-  </si>
-  <si>
     <t>LCSC/MOQ/5 Boards</t>
   </si>
   <si>
@@ -855,6 +852,9 @@
   </si>
   <si>
     <t>C2935910</t>
+  </si>
+  <si>
+    <t>Quantity (Per Board)</t>
   </si>
 </sst>
 </file>
@@ -1607,12 +1607,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>607218</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>33130</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>19942</xdr:rowOff>
+      <xdr:rowOff>53072</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2438400" cy="1164730"/>
+    <xdr:ext cx="2383009" cy="1089928"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="Picture 8">
@@ -1639,8 +1639,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12590859" y="633114"/>
-          <a:ext cx="2438400" cy="1164730"/>
+          <a:off x="12647543" y="657702"/>
+          <a:ext cx="2383009" cy="1089928"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1926,8 +1926,8 @@
     <col min="6" max="6" width="29.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.85546875" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="19.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2077,10 +2077,10 @@
         <v>185</v>
       </c>
       <c r="J9" s="62" t="s">
+        <v>274</v>
+      </c>
+      <c r="K9" s="30" t="s">
         <v>216</v>
-      </c>
-      <c r="K9" s="30" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="38.25" x14ac:dyDescent="0.25">
@@ -2133,13 +2133,13 @@
         <v>102</v>
       </c>
       <c r="F11" s="53" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G11" s="44" t="s">
         <v>157</v>
       </c>
       <c r="H11" s="53" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="I11" s="44" t="s">
         <v>187</v>
@@ -2173,7 +2173,7 @@
         <v>158</v>
       </c>
       <c r="H12" s="54" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I12" s="45" t="s">
         <v>188</v>
@@ -2207,7 +2207,7 @@
         <v>159</v>
       </c>
       <c r="H13" s="53" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I13" s="44" t="s">
         <v>189</v>
@@ -2241,7 +2241,7 @@
         <v>160</v>
       </c>
       <c r="H14" s="54" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I14" s="45" t="s">
         <v>190</v>
@@ -2275,7 +2275,7 @@
         <v>159</v>
       </c>
       <c r="H15" s="53" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I15" s="44" t="s">
         <v>191</v>
@@ -2309,7 +2309,7 @@
         <v>157</v>
       </c>
       <c r="H16" s="54" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I16" s="45" t="s">
         <v>192</v>
@@ -2331,19 +2331,19 @@
         <v>18</v>
       </c>
       <c r="D17" s="53" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E17" s="44" t="s">
         <v>102</v>
       </c>
       <c r="F17" s="44" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G17" s="44" t="s">
         <v>159</v>
       </c>
       <c r="H17" s="53" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I17" s="44" t="s">
         <v>193</v>
@@ -2377,7 +2377,7 @@
         <v>157</v>
       </c>
       <c r="H18" s="54" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="I18" s="45" t="s">
         <v>194</v>
@@ -2411,7 +2411,7 @@
         <v>161</v>
       </c>
       <c r="H19" s="53" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I19" s="50" t="s">
         <v>212</v>
@@ -2445,7 +2445,7 @@
         <v>162</v>
       </c>
       <c r="H20" s="54" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I20" s="51" t="s">
         <v>212</v>
@@ -2479,7 +2479,7 @@
         <v>163</v>
       </c>
       <c r="H21" s="53" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I21" s="50" t="s">
         <v>212</v>
@@ -2513,7 +2513,7 @@
         <v>164</v>
       </c>
       <c r="H22" s="54" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I22" s="51" t="s">
         <v>212</v>
@@ -2535,19 +2535,19 @@
         <v>24</v>
       </c>
       <c r="D23" s="44" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E23" s="44" t="s">
         <v>108</v>
       </c>
       <c r="F23" s="50" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G23" s="44" t="s">
+        <v>271</v>
+      </c>
+      <c r="H23" s="53" t="s">
         <v>272</v>
-      </c>
-      <c r="H23" s="53" t="s">
-        <v>273</v>
       </c>
       <c r="I23" s="50" t="s">
         <v>212</v>
@@ -2581,7 +2581,7 @@
         <v>161</v>
       </c>
       <c r="H24" s="54" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="I24" s="51" t="s">
         <v>212</v>
@@ -2603,19 +2603,19 @@
         <v>26</v>
       </c>
       <c r="D25" s="55" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E25" s="44" t="s">
         <v>110</v>
       </c>
       <c r="F25" s="50" t="s">
+        <v>270</v>
+      </c>
+      <c r="G25" s="44" t="s">
         <v>271</v>
       </c>
-      <c r="G25" s="44" t="s">
-        <v>272</v>
-      </c>
       <c r="H25" s="53" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I25" s="50" t="s">
         <v>212</v>
@@ -2649,7 +2649,7 @@
         <v>160</v>
       </c>
       <c r="H26" s="57" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I26" s="45" t="s">
         <v>195</v>
@@ -2683,7 +2683,7 @@
         <v>165</v>
       </c>
       <c r="H27" s="53" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I27" s="44" t="s">
         <v>196</v>
@@ -2717,7 +2717,7 @@
         <v>166</v>
       </c>
       <c r="H28" s="54" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="I28" s="45" t="s">
         <v>196</v>
@@ -2751,7 +2751,7 @@
         <v>167</v>
       </c>
       <c r="H29" s="53" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I29" s="44" t="s">
         <v>197</v>
@@ -2785,7 +2785,7 @@
         <v>157</v>
       </c>
       <c r="H30" s="54" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="I30" s="45" t="s">
         <v>198</v>
@@ -2819,7 +2819,7 @@
         <v>157</v>
       </c>
       <c r="H31" s="53" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I31" s="50" t="s">
         <v>213</v>
@@ -2853,7 +2853,7 @@
         <v>168</v>
       </c>
       <c r="H32" s="54" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I32" s="45" t="s">
         <v>199</v>
@@ -2881,13 +2881,13 @@
         <v>117</v>
       </c>
       <c r="F33" s="53" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G33" s="44" t="s">
         <v>169</v>
       </c>
       <c r="H33" s="53" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I33" s="50" t="s">
         <v>213</v>
@@ -2915,13 +2915,13 @@
         <v>117</v>
       </c>
       <c r="F34" s="54" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G34" s="45" t="s">
         <v>169</v>
       </c>
       <c r="H34" s="54" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="I34" s="51" t="s">
         <v>213</v>
@@ -2955,7 +2955,7 @@
         <v>170</v>
       </c>
       <c r="H35" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I35" s="44" t="s">
         <v>200</v>
@@ -2977,19 +2977,19 @@
         <v>37</v>
       </c>
       <c r="D36" s="54" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E36" s="45" t="s">
         <v>119</v>
       </c>
       <c r="F36" s="45" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="G36" s="45" t="s">
         <v>159</v>
       </c>
       <c r="H36" s="54" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="I36" s="45" t="s">
         <v>201</v>
@@ -3023,7 +3023,7 @@
         <v>159</v>
       </c>
       <c r="H37" s="53" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I37" s="44" t="s">
         <v>202</v>
@@ -3057,7 +3057,7 @@
         <v>171</v>
       </c>
       <c r="H38" s="54" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I38" s="45" t="s">
         <v>203</v>
@@ -3085,13 +3085,13 @@
         <v>119</v>
       </c>
       <c r="F39" s="53" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="G39" s="44" t="s">
         <v>172</v>
       </c>
       <c r="H39" s="53" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I39" s="44" t="s">
         <v>204</v>
@@ -3119,13 +3119,13 @@
         <v>119</v>
       </c>
       <c r="F40" s="54" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G40" s="45" t="s">
         <v>172</v>
       </c>
       <c r="H40" s="54" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="I40" s="45" t="s">
         <v>205</v>
@@ -3153,13 +3153,13 @@
         <v>118</v>
       </c>
       <c r="F41" s="53" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G41" s="44" t="s">
         <v>173</v>
       </c>
       <c r="H41" s="53" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="I41" s="44" t="s">
         <v>206</v>
@@ -3193,7 +3193,7 @@
         <v>159</v>
       </c>
       <c r="H42" s="54" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I42" s="45" t="s">
         <v>207</v>
@@ -3227,7 +3227,7 @@
         <v>213</v>
       </c>
       <c r="H43" s="55" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I43" s="50" t="s">
         <v>213</v>
@@ -3261,7 +3261,7 @@
         <v>174</v>
       </c>
       <c r="H44" s="54" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="I44" s="51" t="s">
         <v>213</v>
@@ -3295,7 +3295,7 @@
         <v>175</v>
       </c>
       <c r="H45" s="55" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I45" s="50" t="s">
         <v>213</v>
@@ -3329,7 +3329,7 @@
         <v>176</v>
       </c>
       <c r="H46" s="54" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="I46" s="51" t="s">
         <v>213</v>
@@ -3363,7 +3363,7 @@
         <v>177</v>
       </c>
       <c r="H47" s="55" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I47" s="50" t="s">
         <v>213</v>
@@ -3397,7 +3397,7 @@
         <v>178</v>
       </c>
       <c r="H48" s="54" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="I48" s="51" t="s">
         <v>213</v>
@@ -3465,7 +3465,7 @@
         <v>180</v>
       </c>
       <c r="H50" s="54" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I50" s="51" t="s">
         <v>213</v>
@@ -3499,7 +3499,7 @@
         <v>181</v>
       </c>
       <c r="H51" s="53" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I51" s="50" t="s">
         <v>213</v>
@@ -3533,7 +3533,7 @@
         <v>182</v>
       </c>
       <c r="H52" s="54" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="I52" s="51" t="s">
         <v>213</v>
@@ -3567,7 +3567,7 @@
         <v>183</v>
       </c>
       <c r="H53" s="53" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I53" s="44" t="s">
         <v>208</v>
@@ -3601,7 +3601,7 @@
         <v>183</v>
       </c>
       <c r="H54" s="54" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I54" s="45" t="s">
         <v>209</v>
@@ -3635,7 +3635,7 @@
         <v>184</v>
       </c>
       <c r="H55" s="56" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="I55" s="60" t="s">
         <v>210</v>

</xml_diff>